<commit_message>
chore(auto): hourly snapshot 2026-06-29 13:30 KST
</commit_message>
<xml_diff>
--- a/outputs/blog-published-ranks/target-blog-posts-keyword-sheet-mar-jun-all-with-rank-20260629.xlsx
+++ b/outputs/blog-published-ranks/target-blog-posts-keyword-sheet-mar-jun-all-with-rank-20260629.xlsx
@@ -13,8 +13,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="호이호이" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'제이제이'!$A$1:$E$153</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'철인삼남매'!$A$1:$E$87</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'제이제이'!$A$1:$E$147</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'철인삼남매'!$A$1:$E$86</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'사랑채마켓'!$A$1:$E$72</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'호이호이'!$A$1:$E$60</definedName>
   </definedNames>
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F153"/>
+  <dimension ref="A1:F147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -482,7 +482,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>가경동 맛</t>
+          <t>창심관 청주점</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -550,7 +550,9 @@
       <c r="E4" t="n">
         <v>1</v>
       </c>
-      <c r="F4" t="inlineStr"/>
+      <c r="F4" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -560,7 +562,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>곳만</t>
+          <t>카츠바이콘반</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1512,7 +1514,9 @@
       <c r="E41" t="n">
         <v>1</v>
       </c>
-      <c r="F41" t="inlineStr"/>
+      <c r="F41" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1699,22 +1703,22 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224290292557</t>
+          <t>https://blog.naver.com/dnation09/224292462021</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>산호초 논현점</t>
+          <t>월가갈비</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>논현역 회식</t>
+          <t>덕수궁 맛집</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>2026. 5. 19.</t>
+          <t>2026. 5. 21.</t>
         </is>
       </c>
       <c r="E49" t="n">
@@ -1725,38 +1729,38 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224292462021</t>
+          <t>https://blog.naver.com/dnation09/224325754519</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>월가갈비</t>
+          <t>무등소갈비 대구메리어트점</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>덕수궁 맛집</t>
+          <t>동대구역 맛집</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>2026. 5. 21.</t>
+          <t>2026. 6. 24.</t>
         </is>
       </c>
       <c r="E50" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224325754519</t>
+          <t>https://blog.naver.com/dnation09/224303820166</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>무등소갈비 대구메리어트점</t>
+          <t>우야지막창 동대구역점</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -1766,7 +1770,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>2026. 6. 24.</t>
+          <t>2026. 6. 2.</t>
         </is>
       </c>
       <c r="E51" t="n">
@@ -1777,22 +1781,22 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224303820166</t>
+          <t>https://blog.naver.com/dnation09/224306789336</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>우야지막창 동대구역점</t>
+          <t>창심관 동탄</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>동대구역 맛집</t>
+          <t>동탄 고깃집</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>2026. 6. 2.</t>
+          <t>2026. 6. 7.</t>
         </is>
       </c>
       <c r="E52" t="n">
@@ -1803,7 +1807,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224306789336</t>
+          <t>https://blog.naver.com/dnation09/224234122983</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1818,7 +1822,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>2026. 6. 7.</t>
+          <t>2026. 3. 30.</t>
         </is>
       </c>
       <c r="E53" t="n">
@@ -1829,7 +1833,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224234122983</t>
+          <t>https://blog.naver.com/dnation09/224310631049</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1839,23 +1843,23 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>동탄 고깃집</t>
+          <t>동탄 룸식당</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>2026. 3. 30.</t>
+          <t>2026. 6. 9.</t>
         </is>
       </c>
       <c r="E54" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224310631049</t>
+          <t>https://blog.naver.com/dnation09/224328009168</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1865,23 +1869,23 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>동탄 룸식당</t>
+          <t>동탄맛집</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>2026. 6. 9.</t>
+          <t>2026. 6. 28.</t>
         </is>
       </c>
       <c r="E55" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224328009168</t>
+          <t>https://blog.naver.com/dnation09/224316459013</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1896,7 +1900,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>2026. 6. 28.</t>
+          <t>2026. 6. 15.</t>
         </is>
       </c>
       <c r="E56" t="n">
@@ -1907,38 +1911,38 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224316459013</t>
+          <t>https://blog.naver.com/dnation09/224320867304</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>창심관 동탄</t>
+          <t>상록회관연탄구이 문래점</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>동탄맛집</t>
+          <t>문래 맛집</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>2026. 6. 15.</t>
+          <t>2026. 6. 21.</t>
         </is>
       </c>
       <c r="E57" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224320867304</t>
+          <t>https://blog.naver.com/dnation09/224313039184</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>상록회관연탄구이 문래점</t>
+          <t>우시이토 문래점</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -1948,7 +1952,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>2026. 6. 21.</t>
+          <t>2026. 6. 11.</t>
         </is>
       </c>
       <c r="E58" t="n">
@@ -1959,7 +1963,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224313039184</t>
+          <t>https://blog.naver.com/dnation09/224287529300</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1974,7 +1978,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>2026. 6. 11.</t>
+          <t>2026. 5. 16.</t>
         </is>
       </c>
       <c r="E59" t="n">
@@ -1985,22 +1989,22 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224287529300</t>
+          <t>https://blog.naver.com/dnation09/224324600267</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>우시이토 문래점</t>
+          <t>일편등심 마곡발산점</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>문래 맛집</t>
+          <t>발산역맛집</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>2026. 5. 16.</t>
+          <t>2026. 6. 23.</t>
         </is>
       </c>
       <c r="E60" t="n">
@@ -2011,33 +2015,33 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224269314812</t>
+          <t>https://blog.naver.com/dnation09/224313871692</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>으로 변경한</t>
+          <t>일편등심 마곡발산점</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>발산맛집</t>
+          <t>발산역맛집</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>2026. 4. 30.</t>
+          <t>2026. 6. 14.</t>
         </is>
       </c>
       <c r="E61" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224324600267</t>
+          <t>https://blog.naver.com/dnation09/224276592506</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2052,7 +2056,7 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>2026. 6. 23.</t>
+          <t>2026. 5. 6.</t>
         </is>
       </c>
       <c r="E62" t="n">
@@ -2063,100 +2067,102 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224313871692</t>
+          <t>https://blog.naver.com/dnation09/224261323389</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>일편등심 마곡발산점</t>
+          <t>굽돌집 잠실방이직영점</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>발산역맛집</t>
+          <t>방이동맛집</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>2026. 6. 14.</t>
+          <t>2026. 4. 22.</t>
         </is>
       </c>
       <c r="E63" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224276592506</t>
+          <t>https://blog.naver.com/dnation09/224324583242</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>일편등심 마곡발산점</t>
+          <t>굽돌집 잠실방이직영점</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>발산역맛집</t>
+          <t>방이동 회식</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>2026. 5. 6.</t>
+          <t>2026. 6. 23.</t>
         </is>
       </c>
       <c r="E64" t="n">
-        <v>3</v>
-      </c>
-      <c r="F64" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="F64" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224261323389</t>
+          <t>https://blog.naver.com/dnation09/224305692568</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>굽돌집 잠실방이직영점</t>
+          <t>먹자골목 맛집 초원소금구</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>방이동맛집</t>
+          <t>방이동 회식</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>2026. 4. 22.</t>
+          <t>2026. 6. 4.</t>
         </is>
       </c>
       <c r="E65" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224324583242</t>
+          <t>https://blog.naver.com/dnation09/224327138087</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>굽돌집 잠실방이직영점</t>
+          <t>맵시 낙지 백운호수직영점</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>방이동 회식</t>
+          <t>백운호수맛집</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>2026. 6. 23.</t>
+          <t>2026. 6. 26.</t>
         </is>
       </c>
       <c r="E66" t="n">
@@ -2167,22 +2173,22 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224305692568</t>
+          <t>https://blog.naver.com/dnation09/224271764399</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>먹자골목 맛집 초원소금구</t>
+          <t>맵시 낙지 백운호수직영점</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>방이동 회식</t>
+          <t>백운호수맛집</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>2026. 6. 4.</t>
+          <t>2026. 5. 2.</t>
         </is>
       </c>
       <c r="E67" t="n">
@@ -2193,74 +2199,74 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224327138087</t>
+          <t>https://blog.naver.com/dnation09/224318768054</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>맵시 낙지 백운호수직영점</t>
+          <t>낙지마실</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>백운호수맛집</t>
+          <t>보문단지 맛집</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>2026. 6. 26.</t>
+          <t>2026. 6. 17.</t>
         </is>
       </c>
       <c r="E68" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224271764399</t>
+          <t>https://blog.naver.com/dnation09/224236771508</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>맵시 낙지 백운호수직영점</t>
+          <t>우심재</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>백운호수맛집</t>
+          <t>부천 상견례</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>2026. 5. 2.</t>
+          <t>2026. 4. 1.</t>
         </is>
       </c>
       <c r="E69" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224318768054</t>
+          <t>https://blog.naver.com/dnation09/224327821259</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>낙지마실</t>
+          <t>대수부훠궈 부천점</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>보문단지 맛집</t>
+          <t>부천역 맛집</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>2026. 6. 17.</t>
+          <t>2026. 6. 27.</t>
         </is>
       </c>
       <c r="E70" t="n">
@@ -2271,22 +2277,22 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224236771508</t>
+          <t>https://blog.naver.com/dnation09/224263478518</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>우심재</t>
+          <t>사당 광안리 사당본점</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>부천 상견례</t>
+          <t>사당 술집</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>2026. 4. 1.</t>
+          <t>2026. 4. 26.</t>
         </is>
       </c>
       <c r="E71" t="n">
@@ -2297,22 +2303,22 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224327821259</t>
+          <t>https://blog.naver.com/dnation09/224276597884</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>대수부훠궈 부천점</t>
+          <t>사당 광안리 사당본점</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>부천역 맛집</t>
+          <t>사당역 술집</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>2026. 6. 27.</t>
+          <t>2026. 5. 6.</t>
         </is>
       </c>
       <c r="E72" t="n">
@@ -2323,22 +2329,22 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224263478518</t>
+          <t>https://blog.naver.com/dnation09/224311599619</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>사당 광안리 사당본점</t>
+          <t>워낭 사당본점</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>사당 술집</t>
+          <t>사당역 이자카야</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>2026. 4. 26.</t>
+          <t>2026. 6. 10.</t>
         </is>
       </c>
       <c r="E73" t="n">
@@ -2349,22 +2355,22 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224276597884</t>
+          <t>https://blog.naver.com/dnation09/224281950924</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>사당 광안리 사당본점</t>
+          <t>창심관</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>사당역 술집</t>
+          <t>산남동 맛집</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>2026. 5. 6.</t>
+          <t>2026. 5. 11.</t>
         </is>
       </c>
       <c r="E74" t="n">
@@ -2375,22 +2381,22 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224311599619</t>
+          <t>https://blog.naver.com/dnation09/224302801612</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>워낭 사당본점</t>
+          <t>충정화로</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>사당역 이자카야</t>
+          <t>서대문역 맛집</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>2026. 6. 10.</t>
+          <t>2026. 6. 1.</t>
         </is>
       </c>
       <c r="E75" t="n">
@@ -2401,22 +2407,22 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224281950924</t>
+          <t>https://blog.naver.com/dnation09/224276601800</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>성안길 맛</t>
+          <t>우동키노야 서현점</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>산남동 맛집</t>
+          <t>서현 맛집</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>2026. 5. 11.</t>
+          <t>2026. 5. 6.</t>
         </is>
       </c>
       <c r="E76" t="n">
@@ -2427,22 +2433,22 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224302801612</t>
+          <t>https://blog.naver.com/dnation09/224262620446</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>충정화로</t>
+          <t>우와해 선릉본점</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>서대문역 맛집</t>
+          <t>선릉역 맛집</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>2026. 6. 1.</t>
+          <t>2026. 4. 24.</t>
         </is>
       </c>
       <c r="E77" t="n">
@@ -2453,22 +2459,22 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224276601800</t>
+          <t>https://blog.naver.com/dnation09/224218804445</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>우동키노야 서현점</t>
+          <t>성수다락</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>서현 맛집</t>
+          <t>성수동 맛집</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>2026. 5. 6.</t>
+          <t>2026. 3. 19.</t>
         </is>
       </c>
       <c r="E78" t="n">
@@ -2479,74 +2485,74 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224262620446</t>
+          <t>https://blog.naver.com/dnation09/224326692276</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>우와해 선릉본점</t>
+          <t>우동키노야 성수점</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>선릉역 맛집</t>
+          <t>성수 맛집</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>2026. 4. 24.</t>
+          <t>2026. 6. 25.</t>
         </is>
       </c>
       <c r="E79" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224274394638</t>
+          <t>https://blog.naver.com/dnation09/224319903491</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>우와해 선릉본점</t>
+          <t>우동키노야 성수점</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>선릉역 회식</t>
+          <t>성수 맛집</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>2026. 5. 4.</t>
+          <t>2026. 6. 19.</t>
         </is>
       </c>
       <c r="E80" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224218804445</t>
+          <t>https://blog.naver.com/dnation09/224306815930</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>성수다락</t>
+          <t>오밀 성수</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>성수동 맛집</t>
+          <t>성수역 데이트</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>2026. 3. 19.</t>
+          <t>2026. 6. 7.</t>
         </is>
       </c>
       <c r="E81" t="n">
@@ -2557,48 +2563,48 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224326692276</t>
+          <t>https://blog.naver.com/dnation09/224311036827</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>우동키노야 성수점</t>
+          <t>소보루 성심당</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>성수 맛집</t>
+          <t>성심당</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>2026. 6. 25.</t>
+          <t>2026. 6. 9.</t>
         </is>
       </c>
       <c r="E82" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224319903491</t>
+          <t>https://blog.naver.com/dnation09/224325766211</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>우동키노야 성수점</t>
+          <t>고담현불고기 해운대센텀시티점</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>성수 맛집</t>
+          <t>센텀맛집</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>2026. 6. 19.</t>
+          <t>2026. 6. 24.</t>
         </is>
       </c>
       <c r="E83" t="n">
@@ -2609,48 +2615,48 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224306815930</t>
+          <t>https://blog.naver.com/dnation09/224279082523</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>오밀 성수</t>
+          <t>고담현불고기 해운대센텀시티점</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>성수역 데이트</t>
+          <t>센텀맛집</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>2026. 6. 7.</t>
+          <t>2026. 5. 9.</t>
         </is>
       </c>
       <c r="E84" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224311036827</t>
+          <t>https://blog.naver.com/dnation09/224254689483</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>소보루 성심당</t>
+          <t>옛 고을순두부</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>성심당</t>
+          <t>속초맛집</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>2026. 6. 9.</t>
+          <t>2026. 4. 16.</t>
         </is>
       </c>
       <c r="E85" t="n">
@@ -2661,74 +2667,74 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224325766211</t>
+          <t>https://blog.naver.com/dnation09/224298984152</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>고담현불고기 해운대센텀시티점</t>
+          <t>청초수물회 속초</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>센텀맛집</t>
+          <t>속초 해수욕장 맛집</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>2026. 6. 24.</t>
+          <t>2026. 5. 28.</t>
         </is>
       </c>
       <c r="E86" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224279082523</t>
+          <t>https://blog.naver.com/dnation09/224326702798</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>고담현불고기 해운대센텀시티점</t>
+          <t>럭키족발 송도점</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>센텀맛집</t>
+          <t>송도 맛집</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>2026. 5. 9.</t>
+          <t>2026. 6. 25.</t>
         </is>
       </c>
       <c r="E87" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224254689483</t>
+          <t>https://blog.naver.com/dnation09/224261008327</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>옛 고을순두부</t>
+          <t>백호동태 송도점</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>속초맛집</t>
+          <t>송도 샤브샤브</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>2026. 4. 16.</t>
+          <t>2026. 4. 22.</t>
         </is>
       </c>
       <c r="E88" t="n">
@@ -2739,22 +2745,22 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224260050406</t>
+          <t>https://blog.naver.com/dnation09/224316441821</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>청초수물회 속초본점</t>
+          <t>샤브밀</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>속초 점심</t>
+          <t>수원맛집</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>2026. 4. 21.</t>
+          <t>2026. 6. 15.</t>
         </is>
       </c>
       <c r="E89" t="n">
@@ -2765,22 +2771,22 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224298984152</t>
+          <t>https://blog.naver.com/dnation09/224285429415</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>청초수물회 속초</t>
+          <t>상록회관연탄구이 수원스타필드점</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>속초 해수욕장 맛집</t>
+          <t>수원 스타필드 맛집</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>2026. 5. 28.</t>
+          <t>2026. 5. 14.</t>
         </is>
       </c>
       <c r="E90" t="n">
@@ -2791,59 +2797,59 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224326702798</t>
+          <t>https://blog.naver.com/dnation09/224328005281</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>럭키족발 송도점</t>
+          <t>샤브밀</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>송도 맛집</t>
+          <t>수원역맛집</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>2026. 6. 25.</t>
+          <t>2026. 6. 28.</t>
         </is>
       </c>
       <c r="E91" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224261008327</t>
+          <t>https://blog.naver.com/dnation09/224320846415</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>백호동태 송도점</t>
+          <t>샤브밀</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>송도 샤브샤브</t>
+          <t>수원역맛집</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>2026. 4. 22.</t>
+          <t>2026. 6. 20.</t>
         </is>
       </c>
       <c r="E92" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224316441821</t>
+          <t>https://blog.naver.com/dnation09/224313855889</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -2853,38 +2859,38 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>수원맛집</t>
+          <t>수원역맛집</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>2026. 6. 15.</t>
+          <t>2026. 6. 12.</t>
         </is>
       </c>
       <c r="E93" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224285429415</t>
+          <t>https://blog.naver.com/dnation09/224305691521</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>상록회관연탄구이 수원스타필드점</t>
+          <t>멘쿠도</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>수원 스타필드 맛집</t>
+          <t>신논현 데이트</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>2026. 5. 14.</t>
+          <t>2026. 6. 4.</t>
         </is>
       </c>
       <c r="E94" t="n">
@@ -2895,100 +2901,100 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224328005281</t>
+          <t>https://blog.naver.com/dnation09/224266817285</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>샤브밀</t>
+          <t>서울집</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>수원역맛집</t>
+          <t>신논현 맛집</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>2026. 6. 28.</t>
+          <t>2026. 4. 28.</t>
         </is>
       </c>
       <c r="E95" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224320846415</t>
+          <t>https://blog.naver.com/dnation09/224266797516</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>샤브밀</t>
+          <t>우동키노야 강남신논현역점</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>수원역맛집</t>
+          <t>신논현역 맛집</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>2026. 6. 20.</t>
+          <t>2026. 4. 27.</t>
         </is>
       </c>
       <c r="E96" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224313855889</t>
+          <t>https://blog.naver.com/dnation09/224323372135</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>샤브밀</t>
+          <t>우동키노야 신용산본점</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>수원역맛집</t>
+          <t>신용산 맛집</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>2026. 6. 12.</t>
+          <t>2026. 6. 22.</t>
         </is>
       </c>
       <c r="E97" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224305691521</t>
+          <t>https://blog.naver.com/dnation09/224313041293</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>멘쿠도</t>
+          <t>산산바베큐치킨 신촌본점</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>신논현 데이트</t>
+          <t>신촌 술집</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>2026. 6. 4.</t>
+          <t>2026. 6. 11.</t>
         </is>
       </c>
       <c r="E98" t="n">
@@ -2999,22 +3005,22 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224266817285</t>
+          <t>https://blog.naver.com/dnation09/224327134620</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>서울집</t>
+          <t>회삼춘</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>신논현 맛집</t>
+          <t>아산맛집</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>2026. 4. 28.</t>
+          <t>2026. 6. 26.</t>
         </is>
       </c>
       <c r="E99" t="n">
@@ -3025,74 +3031,74 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224266797516</t>
+          <t>https://blog.naver.com/dnation09/224327825102</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>우동키노야 강남신논현역점</t>
+          <t>라성돌판요리</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>신논현역 맛집</t>
+          <t>안산맛집</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>2026. 4. 27.</t>
+          <t>2026. 6. 27.</t>
         </is>
       </c>
       <c r="E100" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224262624419</t>
+          <t>https://blog.naver.com/dnation09/224317481816</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>산호초 논현점</t>
+          <t>라성돌판요리</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>신논현 횟집</t>
+          <t>안산맛집</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>2026. 4. 24.</t>
+          <t>2026. 6. 16.</t>
         </is>
       </c>
       <c r="E101" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224323372135</t>
+          <t>https://blog.naver.com/dnation09/224326698496</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>우동키노야 신용산본점</t>
+          <t>델리커리 안양엔터식스점</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>신용산 맛집</t>
+          <t>안양역맛집</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>2026. 6. 22.</t>
+          <t>2026. 6. 25.</t>
         </is>
       </c>
       <c r="E102" t="n">
@@ -3103,22 +3109,22 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224313041293</t>
+          <t>https://blog.naver.com/dnation09/224305759738</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>산산바베큐치킨 신촌본점</t>
+          <t>가야부처스 양산점</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>신촌 술집</t>
+          <t>양산 맛집</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>2026. 6. 11.</t>
+          <t>2026. 6. 4.</t>
         </is>
       </c>
       <c r="E103" t="n">
@@ -3129,22 +3135,22 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224327134620</t>
+          <t>https://blog.naver.com/dnation09/224239401838</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>회삼춘</t>
+          <t>상록회관연탄구이 여수여서점</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>아산맛집</t>
+          <t>여수 고기집</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>2026. 6. 26.</t>
+          <t>2026. 4. 5.</t>
         </is>
       </c>
       <c r="E104" t="n">
@@ -3155,74 +3161,74 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224327825102</t>
+          <t>https://blog.naver.com/dnation09/224218811093</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>라성돌판요리</t>
+          <t>부일갈비</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>안산맛집</t>
+          <t>여의도 맛집</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>2026. 6. 27.</t>
+          <t>2026. 3. 21.</t>
         </is>
       </c>
       <c r="E105" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224317481816</t>
+          <t>https://blog.naver.com/dnation09/224266812269</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>라성돌판요리</t>
+          <t>사위식당 여의도점</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>안산맛집</t>
+          <t>여의도 점심 맛집</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>2026. 6. 16.</t>
+          <t>2026. 4. 28.</t>
         </is>
       </c>
       <c r="E106" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224326698496</t>
+          <t>https://blog.naver.com/dnation09/224297941884</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>델리커리 안양엔터식스점</t>
+          <t>명장갈비 오송점</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>안양역맛집</t>
+          <t>오송 회식</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>2026. 6. 25.</t>
+          <t>2026. 5. 27.</t>
         </is>
       </c>
       <c r="E107" t="n">
@@ -3233,22 +3239,22 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224305759738</t>
+          <t>https://blog.naver.com/dnation09/224320853609</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>가야부처스 양산점</t>
+          <t>홍홍대패 오창점</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>양산 맛집</t>
+          <t>오창 맛집</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>2026. 6. 4.</t>
+          <t>2026. 6. 20.</t>
         </is>
       </c>
       <c r="E108" t="n">
@@ -3259,199 +3265,201 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224239401838</t>
+          <t>https://blog.naver.com/dnation09/224323368956</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>상록회관연탄구이 여수여서점</t>
+          <t>우동키노야 신용산본점</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>여수 고기집</t>
+          <t>용산 맛집</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>2026. 4. 5.</t>
+          <t>2026. 6. 22.</t>
         </is>
       </c>
       <c r="E109" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224218811093</t>
+          <t>https://blog.naver.com/dnation09/224318771810</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>곳만</t>
+          <t>우동키노야 신용산본점</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>여의도 맛집</t>
+          <t>용산 맛집</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>2026. 3. 21.</t>
+          <t>2026. 6. 17.</t>
         </is>
       </c>
       <c r="E110" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224266812269</t>
+          <t>https://blog.naver.com/dnation09/224319912821</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>사위식당 여의도점</t>
+          <t>바램 청주 율량점</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>여의도 점심 맛집</t>
+          <t>율량동 맛집</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>2026. 4. 28.</t>
+          <t>2026. 6. 19.</t>
         </is>
       </c>
       <c r="E111" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224297941884</t>
+          <t>https://blog.naver.com/dnation09/224316450629</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>명장갈비 오송점</t>
+          <t>창심관 율량점</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>오송 회식</t>
+          <t>율량동 맛집</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>2026. 5. 27.</t>
+          <t>2026. 6. 15.</t>
         </is>
       </c>
       <c r="E112" t="n">
-        <v>1</v>
-      </c>
-      <c r="F112" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="F112" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224320853609</t>
+          <t>https://blog.naver.com/dnation09/224303975835</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>홍홍대패 오창점</t>
+          <t>바램 청주 율량점</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>오창 맛집</t>
+          <t>율량동 맛집</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>2026. 6. 20.</t>
+          <t>2026. 6. 3.</t>
         </is>
       </c>
       <c r="E113" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224323368956</t>
+          <t>https://blog.naver.com/dnation09/224290289664</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>우동키노야 신용산본점</t>
+          <t>창심관 율량점</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>용산 맛집</t>
+          <t>율량동 맛집</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>2026. 6. 22.</t>
+          <t>2026. 5. 19.</t>
         </is>
       </c>
       <c r="E114" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224318771810</t>
+          <t>https://blog.naver.com/dnation09/224303840498</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>우동키노야 신용산본점</t>
+          <t>보성갈비</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>용산 맛집</t>
+          <t>율량동 회식</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>2026. 6. 17.</t>
+          <t>2026. 6. 2.</t>
         </is>
       </c>
       <c r="E115" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224319912821</t>
+          <t>https://blog.naver.com/dnation09/224319908213</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>바램 청주 율량점</t>
+          <t>금성회관 을지로점</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>율량동 맛집</t>
+          <t>을지로 맛집</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -3460,133 +3468,133 @@
         </is>
       </c>
       <c r="E116" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224316450629</t>
+          <t>https://blog.naver.com/dnation09/224302900830</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>창심관 율량점</t>
+          <t>맵시 낙지 백운호수직영점</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>율량동 맛집</t>
+          <t>의왕롯데아울렛</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>2026. 6. 15.</t>
+          <t>2026. 6. 1.</t>
         </is>
       </c>
       <c r="E117" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224303975835</t>
+          <t>https://blog.naver.com/dnation09/224271767618</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>바램 청주 율량점</t>
+          <t>맵시 낙지 백운호수직영점</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>율량동 맛집</t>
+          <t>의왕롯데아울렛</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>2026. 6. 3.</t>
+          <t>2026. 5. 2.</t>
         </is>
       </c>
       <c r="E118" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224290289664</t>
+          <t>https://blog.naver.com/dnation09/224302851182</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>창심관 율량점</t>
+          <t>항아리정육식당 의정부</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>율량동 맛집</t>
+          <t>의정부역 맛집</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>2026. 5. 19.</t>
+          <t>2026. 6. 1.</t>
         </is>
       </c>
       <c r="E119" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224303840498</t>
+          <t>https://blog.naver.com/dnation09/224232751060</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>보성갈비</t>
+          <t>항아리정육식당 의정부</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>율량동 회식</t>
+          <t>의정부역 맛집</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>2026. 6. 2.</t>
+          <t>2026. 3. 28.</t>
         </is>
       </c>
       <c r="E120" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224319908213</t>
+          <t>https://blog.naver.com/dnation09/224218814222</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>금성회관 을지로점</t>
+          <t>소와나</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>을지로 맛집</t>
+          <t>이태원맛집</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>2026. 6. 19.</t>
+          <t>2026. 3. 22.</t>
         </is>
       </c>
       <c r="E121" t="n">
@@ -3597,22 +3605,22 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224302900830</t>
+          <t>https://blog.naver.com/dnation09/224327130461</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>맵시 낙지 백운호수직영점</t>
+          <t>곱따 일산</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>의왕롯데아울렛</t>
+          <t>일산 맛집</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>2026. 6. 1.</t>
+          <t>2026. 6. 26.</t>
         </is>
       </c>
       <c r="E122" t="n">
@@ -3623,22 +3631,22 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224271767618</t>
+          <t>https://blog.naver.com/dnation09/224319895024</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>맵시 낙지 백운호수직영점</t>
+          <t>곱따 일산</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>의왕롯데아울렛</t>
+          <t>일산 맛집</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>2026. 5. 2.</t>
+          <t>2026. 6. 18.</t>
         </is>
       </c>
       <c r="E123" t="n">
@@ -3649,74 +3657,74 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224302851182</t>
+          <t>https://blog.naver.com/dnation09/224218807620</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>항아리정육식당 의정부</t>
+          <t>라쿤피자 잠실</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>의정부역 맛집</t>
+          <t>잠실 맛집</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>2026. 6. 1.</t>
+          <t>2026. 3. 20.</t>
         </is>
       </c>
       <c r="E124" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224232751060</t>
+          <t>https://blog.naver.com/dnation09/224218801341</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>항아리정육식당 의정부</t>
+          <t>샤브가든 종로 타워점</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>의정부역 맛집</t>
+          <t>종로 맛집</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>2026. 3. 28.</t>
+          <t>2026. 3. 18.</t>
         </is>
       </c>
       <c r="E125" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224218814222</t>
+          <t>https://blog.naver.com/dnation09/224222427215</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>7곳, 광고 아님 내돈내산 후기만 모았어요</t>
+          <t>무등소갈비 첨단본점</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>이태원맛집</t>
+          <t>첨단맛집</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>2026. 3. 22.</t>
+          <t>2026. 3. 19.</t>
         </is>
       </c>
       <c r="E126" t="n">
@@ -3727,22 +3735,22 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224327130461</t>
+          <t>https://blog.naver.com/dnation09/224313849939</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>곱따 일산</t>
+          <t>아키아키</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>일산 맛집</t>
+          <t>청주맛집</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>2026. 6. 26.</t>
+          <t>2026. 6. 12.</t>
         </is>
       </c>
       <c r="E127" t="n">
@@ -3753,22 +3761,22 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224319895024</t>
+          <t>https://blog.naver.com/dnation09/224311784919</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>곱따 일산</t>
+          <t>창심관 율량점</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>일산 맛집</t>
+          <t>청주맛집</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>2026. 6. 18.</t>
+          <t>2026. 6. 11.</t>
         </is>
       </c>
       <c r="E128" t="n">
@@ -3779,85 +3787,87 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224218807620</t>
+          <t>https://blog.naver.com/dnation09/224324587645</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>라쿤피자 잠실</t>
+          <t>대구왕뽈때기청주봉명점</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>잠실 맛집</t>
+          <t>청주 봉명동 맛집</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>2026. 3. 20.</t>
+          <t>2026. 6. 23.</t>
         </is>
       </c>
       <c r="E129" t="n">
-        <v>1</v>
-      </c>
-      <c r="F129" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="F129" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224218801341</t>
+          <t>https://blog.naver.com/dnation09/224313866635</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>샤브가든 종로 타워점</t>
+          <t>찜요리 매장</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>종로 맛집</t>
+          <t>청주 봉명동 맛집</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>2026. 3. 18.</t>
+          <t>2026. 6. 13.</t>
         </is>
       </c>
       <c r="E130" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224222427215</t>
+          <t>https://blog.naver.com/dnation09/224313852200</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>무등소갈비 첨단본점</t>
+          <t>아키아키</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>첨단맛집</t>
+          <t>청주상견례</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>2026. 3. 19.</t>
+          <t>2026. 6. 12.</t>
         </is>
       </c>
       <c r="E131" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224313849939</t>
+          <t>https://blog.naver.com/dnation09/224285477671</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3867,12 +3877,12 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>청주맛집</t>
+          <t>청주상견례</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>2026. 6. 12.</t>
+          <t>2026. 5. 14.</t>
         </is>
       </c>
       <c r="E132" t="n">
@@ -3883,152 +3893,152 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224311784919</t>
+          <t>https://blog.naver.com/dnation09/224320885611</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>창심관 율량점</t>
+          <t>아키아키</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>청주맛집</t>
+          <t>청주오마카세</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>2026. 6. 11.</t>
+          <t>2026. 6. 20.</t>
         </is>
       </c>
       <c r="E133" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224324587645</t>
+          <t>https://blog.naver.com/dnation09/224313874620</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>대구왕뽈때기청주봉명점</t>
+          <t>황토골 충무로역 본점</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>청주 봉명동 맛집</t>
+          <t>충무로맛집</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>2026. 6. 23.</t>
+          <t>2026. 6. 14.</t>
         </is>
       </c>
       <c r="E134" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224313866635</t>
+          <t>https://blog.naver.com/dnation09/224325770766</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>봉명동 맛</t>
+          <t>사위식당 판교점</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>청주 봉명동 맛집</t>
+          <t>판교맛집</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>2026. 6. 13.</t>
+          <t>2026. 6. 24.</t>
         </is>
       </c>
       <c r="E135" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224293458593</t>
+          <t>https://blog.naver.com/dnation09/224263730051</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>대구왕뽈때기청주봉명점</t>
+          <t>사위식당 판교점</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>청주 봉명동 맛집</t>
+          <t>판교맛집</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>2026. 5. 22.</t>
+          <t>2026. 4. 25.</t>
         </is>
       </c>
       <c r="E136" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224313852200</t>
+          <t>https://blog.naver.com/dnation09/224261734050</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>아키아키</t>
+          <t>백년가돌판짜장짬뽕</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>청주상견례</t>
+          <t>포천맛집</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>2026. 6. 12.</t>
+          <t>2026. 4. 22.</t>
         </is>
       </c>
       <c r="E137" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224285477671</t>
+          <t>https://blog.naver.com/dnation09/224310644613</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>아키아키</t>
+          <t>대동면옥 올림픽공원직영점</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>청주상견례</t>
+          <t>하남 맛집</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>2026. 5. 14.</t>
+          <t>2026. 6. 10.</t>
         </is>
       </c>
       <c r="E138" t="n">
@@ -4039,74 +4049,74 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224320885611</t>
+          <t>https://blog.naver.com/dnation09/224272762515</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>아키아키</t>
+          <t>대동면옥 올림픽공원직영점</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>청주오마카세</t>
+          <t>하남 맛집</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>2026. 6. 20.</t>
+          <t>2026. 5. 3.</t>
         </is>
       </c>
       <c r="E139" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224313874620</t>
+          <t>https://blog.naver.com/dnation09/224326708508</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>황토골 충무로역 본점</t>
+          <t>우동키노야 합정점</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>충무로맛집</t>
+          <t>합정역 맛집</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>2026. 6. 14.</t>
+          <t>2026. 6. 25.</t>
         </is>
       </c>
       <c r="E140" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224325770766</t>
+          <t>https://blog.naver.com/dnation09/224298972701</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>사위식당 판교점</t>
+          <t>우동키노야 합정점</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>판교맛집</t>
+          <t>합정역 맛집</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>2026. 6. 24.</t>
+          <t>2026. 5. 28.</t>
         </is>
       </c>
       <c r="E141" t="n">
@@ -4117,48 +4127,48 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224263730051</t>
+          <t>https://blog.naver.com/dnation09/224292466308</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>사위식당 판교점</t>
+          <t>신사꽃게당 해운대점</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>판교맛집</t>
+          <t>해운대 맛집</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>2026. 4. 25.</t>
+          <t>2026. 5. 22.</t>
         </is>
       </c>
       <c r="E142" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224261734050</t>
+          <t>https://blog.naver.com/dnation09/224310673870</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>어느달에서 포천 맛</t>
+          <t>신사 꽃게당</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>포천맛집</t>
+          <t>해운대 맛집 추천</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>2026. 4. 22.</t>
+          <t>2026. 6. 9.</t>
         </is>
       </c>
       <c r="E143" t="n">
@@ -4169,48 +4179,48 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224310644613</t>
+          <t>https://blog.naver.com/dnation09/224221445105</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>대동면옥 올림픽공원직영점</t>
+          <t>고기꾼 김춘배</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>하남 맛집</t>
+          <t>홍대 고기집</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>2026. 6. 10.</t>
+          <t>2026. 3. 18.</t>
         </is>
       </c>
       <c r="E144" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224272762515</t>
+          <t>https://blog.naver.com/dnation09/224319899827</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>대동면옥 올림픽공원직영점</t>
+          <t>봉림대패 홍대점</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>하남 맛집</t>
+          <t>홍대 맛집</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>2026. 5. 3.</t>
+          <t>2026. 6. 19.</t>
         </is>
       </c>
       <c r="E145" t="n">
@@ -4221,22 +4231,22 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224326708508</t>
+          <t>https://blog.naver.com/dnation09/224214384106</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>우동키노야 합정점</t>
+          <t>쟁반집 8292 홍대점</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>합정역 맛집</t>
+          <t>홍대 맛집</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>2026. 6. 25.</t>
+          <t>2026. 3. 12.</t>
         </is>
       </c>
       <c r="E146" t="n">
@@ -4247,187 +4257,31 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dnation09/224298972701</t>
+          <t>https://blog.naver.com/dnation09/224284164028</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>우동키노야 합정점</t>
+          <t>봉림대패</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>합정역 맛집</t>
+          <t>홍대 점심 맛집</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>2026. 5. 28.</t>
+          <t>2026. 5. 13.</t>
         </is>
       </c>
       <c r="E147" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F147" t="inlineStr"/>
     </row>
-    <row r="148">
-      <c r="A148" t="inlineStr">
-        <is>
-          <t>https://blog.naver.com/dnation09/224292466308</t>
-        </is>
-      </c>
-      <c r="B148" t="inlineStr">
-        <is>
-          <t>신사꽃게당 해운대점</t>
-        </is>
-      </c>
-      <c r="C148" t="inlineStr">
-        <is>
-          <t>해운대 맛집</t>
-        </is>
-      </c>
-      <c r="D148" t="inlineStr">
-        <is>
-          <t>2026. 5. 22.</t>
-        </is>
-      </c>
-      <c r="E148" t="n">
-        <v>1</v>
-      </c>
-      <c r="F148" t="inlineStr"/>
-    </row>
-    <row r="149">
-      <c r="A149" t="inlineStr">
-        <is>
-          <t>https://blog.naver.com/dnation09/224310673870</t>
-        </is>
-      </c>
-      <c r="B149" t="inlineStr">
-        <is>
-          <t>신사 꽃게당</t>
-        </is>
-      </c>
-      <c r="C149" t="inlineStr">
-        <is>
-          <t>해운대 맛집 추천</t>
-        </is>
-      </c>
-      <c r="D149" t="inlineStr">
-        <is>
-          <t>2026. 6. 9.</t>
-        </is>
-      </c>
-      <c r="E149" t="n">
-        <v>1</v>
-      </c>
-      <c r="F149" t="inlineStr"/>
-    </row>
-    <row r="150">
-      <c r="A150" t="inlineStr">
-        <is>
-          <t>https://blog.naver.com/dnation09/224221445105</t>
-        </is>
-      </c>
-      <c r="B150" t="inlineStr">
-        <is>
-          <t>고기꾼 김춘배</t>
-        </is>
-      </c>
-      <c r="C150" t="inlineStr">
-        <is>
-          <t>홍대 고기집</t>
-        </is>
-      </c>
-      <c r="D150" t="inlineStr">
-        <is>
-          <t>2026. 3. 18.</t>
-        </is>
-      </c>
-      <c r="E150" t="n">
-        <v>1</v>
-      </c>
-      <c r="F150" t="inlineStr"/>
-    </row>
-    <row r="151">
-      <c r="A151" t="inlineStr">
-        <is>
-          <t>https://blog.naver.com/dnation09/224319899827</t>
-        </is>
-      </c>
-      <c r="B151" t="inlineStr">
-        <is>
-          <t>봉림대패 홍대점</t>
-        </is>
-      </c>
-      <c r="C151" t="inlineStr">
-        <is>
-          <t>홍대 맛집</t>
-        </is>
-      </c>
-      <c r="D151" t="inlineStr">
-        <is>
-          <t>2026. 6. 19.</t>
-        </is>
-      </c>
-      <c r="E151" t="n">
-        <v>2</v>
-      </c>
-      <c r="F151" t="inlineStr"/>
-    </row>
-    <row r="152">
-      <c r="A152" t="inlineStr">
-        <is>
-          <t>https://blog.naver.com/dnation09/224214384106</t>
-        </is>
-      </c>
-      <c r="B152" t="inlineStr">
-        <is>
-          <t>쟁반집 8292 홍대점</t>
-        </is>
-      </c>
-      <c r="C152" t="inlineStr">
-        <is>
-          <t>홍대 맛집</t>
-        </is>
-      </c>
-      <c r="D152" t="inlineStr">
-        <is>
-          <t>2026. 3. 12.</t>
-        </is>
-      </c>
-      <c r="E152" t="n">
-        <v>2</v>
-      </c>
-      <c r="F152" t="inlineStr"/>
-    </row>
-    <row r="153">
-      <c r="A153" t="inlineStr">
-        <is>
-          <t>https://blog.naver.com/dnation09/224284164028</t>
-        </is>
-      </c>
-      <c r="B153" t="inlineStr">
-        <is>
-          <t>혼밥 맛</t>
-        </is>
-      </c>
-      <c r="C153" t="inlineStr">
-        <is>
-          <t>홍대 점심 맛집</t>
-        </is>
-      </c>
-      <c r="D153" t="inlineStr">
-        <is>
-          <t>2026. 5. 13.</t>
-        </is>
-      </c>
-      <c r="E153" t="n">
-        <v>1</v>
-      </c>
-      <c r="F153" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:E153"/>
+  <autoFilter ref="A1:E147"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4438,7 +4292,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F87"/>
+  <dimension ref="A1:F86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -4484,7 +4338,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224311776276</t>
+          <t>https://blog.naver.com/dreamclock33/224325728678</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -4494,12 +4348,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>강남 룸식당</t>
+          <t>강남역 회식</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026. 6. 11.</t>
+          <t>2026. 6. 24.</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -4510,33 +4364,33 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224325728678</t>
+          <t>https://blog.naver.com/dreamclock33/224320961599</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>육목원</t>
+          <t>대동면옥 강릉본점</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>강남역 회식</t>
+          <t>강릉맛집추천</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026. 6. 24.</t>
+          <t>2026. 6. 20.</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224320961599</t>
+          <t>https://blog.naver.com/dreamclock33/224313953783</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -4551,7 +4405,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026. 6. 20.</t>
+          <t>2026. 6. 13.</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -4562,7 +4416,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224313953783</t>
+          <t>https://blog.naver.com/dreamclock33/224323265067</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -4572,49 +4426,49 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>강릉맛집추천</t>
+          <t>강릉역 맛집</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026. 6. 13.</t>
+          <t>2026. 6. 22.</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224323265067</t>
+          <t>https://blog.naver.com/dreamclock33/224326680294</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>대동면옥 강릉본점</t>
+          <t>우동키노야 건대입구점</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>강릉역 맛집</t>
+          <t>건대 맛집</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026. 6. 22.</t>
+          <t>2026. 6. 25.</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224326680294</t>
+          <t>https://blog.naver.com/dreamclock33/224317889343</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -4629,7 +4483,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026. 6. 25.</t>
+          <t>2026. 6. 16.</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -4640,64 +4494,64 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224317889343</t>
+          <t>https://blog.naver.com/dreamclock33/224318954324</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>우동키노야 건대입구점</t>
+          <t>하나 샤브샤브 광교점</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>건대 맛집</t>
+          <t>광교 맛집</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026. 6. 16.</t>
+          <t>2026. 6. 18.</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224318954324</t>
+          <t>https://blog.naver.com/dreamclock33/224317892495</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>하나 샤브샤브 광교점</t>
+          <t>우동키노야 광안점</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>광교 맛집</t>
+          <t>광안리맛집</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026. 6. 18.</t>
+          <t>2026. 6. 16.</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224317892495</t>
+          <t>https://blog.naver.com/dreamclock33/224313951143</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>우동키노야 광안점</t>
+          <t>청산1954 광안리본점</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -4707,7 +4561,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026. 6. 16.</t>
+          <t>2026. 6. 13.</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -4718,12 +4572,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224313951143</t>
+          <t>https://blog.naver.com/dreamclock33/224305879066</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>청산1954 광안리본점</t>
+          <t>우동키노야 광안점</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -4733,7 +4587,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026. 6. 13.</t>
+          <t>2026. 6. 5.</t>
         </is>
       </c>
       <c r="E11" t="n">
@@ -4744,48 +4598,48 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224305879066</t>
+          <t>https://blog.naver.com/dreamclock33/224327758671</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>우동키노야 광안점</t>
+          <t>카이루 이자까야 광안본점</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>광안리맛집</t>
+          <t>광안리 이자카야</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026. 6. 5.</t>
+          <t>2026. 6. 27.</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224327758671</t>
+          <t>https://blog.naver.com/dreamclock33/224327121087</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>카이루 이자까야 광안본점</t>
+          <t>금목서 광양불고기</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>광안리 이자카야</t>
+          <t>광양 불고기</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026. 6. 27.</t>
+          <t>2026. 6. 26.</t>
         </is>
       </c>
       <c r="E13" t="n">
@@ -4796,17 +4650,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224327121087</t>
+          <t>https://blog.naver.com/dreamclock33/224327113039</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>금목서 광양불고기</t>
+          <t>샤브가든 종로 타워점</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>광양 불고기</t>
+          <t>광화문 맛집</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -4822,22 +4676,22 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224327113039</t>
+          <t>https://blog.naver.com/dreamclock33/224310604861</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>샤브가든 종로 타워점</t>
+          <t>육풍 구로점</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>광화문 맛집</t>
+          <t>구디맛집</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2026. 6. 26.</t>
+          <t>2026. 6. 10.</t>
         </is>
       </c>
       <c r="E15" t="n">
@@ -4848,22 +4702,22 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224310604861</t>
+          <t>https://blog.naver.com/dreamclock33/224310601723</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>육풍 구로점</t>
+          <t>호우양꼬치 구월</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>구디맛집</t>
+          <t>구월동 맛집</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026. 6. 10.</t>
+          <t>2026. 6. 9.</t>
         </is>
       </c>
       <c r="E16" t="n">
@@ -4874,22 +4728,22 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224310601723</t>
+          <t>https://blog.naver.com/dreamclock33/224308008044</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>호우양꼬치 구월</t>
+          <t>청산1954 광안리본점</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>구월동 맛집</t>
+          <t>남천동맛집</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2026. 6. 9.</t>
+          <t>2026. 6. 7.</t>
         </is>
       </c>
       <c r="E17" t="n">
@@ -4900,33 +4754,33 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224308008044</t>
+          <t>https://blog.naver.com/dreamclock33/224320007361</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>청산1954 광안리본점</t>
+          <t>노들솥뚜껑 노량진점</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>남천동맛집</t>
+          <t>노량진맛집</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2026. 6. 7.</t>
+          <t>2026. 6. 19.</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224320007361</t>
+          <t>https://blog.naver.com/dreamclock33/224302843610</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -4941,7 +4795,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2026. 6. 19.</t>
+          <t>2026. 6. 2.</t>
         </is>
       </c>
       <c r="E19" t="n">
@@ -4952,64 +4806,64 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224302843610</t>
+          <t>https://blog.naver.com/dreamclock33/224327815571</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>노들솥뚜껑 노량진점</t>
+          <t>월가갈비</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>노량진맛집</t>
+          <t>덕수궁 맛집</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2026. 6. 2.</t>
+          <t>2026. 6. 27.</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224327815571</t>
+          <t>https://blog.naver.com/dreamclock33/224325734116</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>월가갈비</t>
+          <t>우야지막창 동대구역점</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>덕수궁 맛집</t>
+          <t>동대구역 맛집</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2026. 6. 27.</t>
+          <t>2026. 6. 24.</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224325734116</t>
+          <t>https://blog.naver.com/dreamclock33/224320003433</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>우야지막창 동대구역점</t>
+          <t>무등소갈비 대구메리어트점</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -5019,7 +4873,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2026. 6. 24.</t>
+          <t>2026. 6. 19.</t>
         </is>
       </c>
       <c r="E22" t="n">
@@ -5030,7 +4884,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224320003433</t>
+          <t>https://blog.naver.com/dreamclock33/224313031738</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -5045,7 +4899,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2026. 6. 19.</t>
+          <t>2026. 6. 12.</t>
         </is>
       </c>
       <c r="E23" t="n">
@@ -5056,7 +4910,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224313031738</t>
+          <t>https://blog.naver.com/dreamclock33/224302839580</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -5071,7 +4925,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>2026. 6. 12.</t>
+          <t>2026. 6. 2.</t>
         </is>
       </c>
       <c r="E24" t="n">
@@ -5082,33 +4936,33 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224302839580</t>
+          <t>https://blog.naver.com/dreamclock33/224327999984</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>무등소갈비 대구메리어트점</t>
+          <t>창심관 동탄</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>동대구역 맛집</t>
+          <t>동탄맛집</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2026. 6. 2.</t>
+          <t>2026. 6. 28.</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224327999984</t>
+          <t>https://blog.naver.com/dreamclock33/224313948831</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -5123,7 +4977,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>2026. 6. 28.</t>
+          <t>2026. 6. 13.</t>
         </is>
       </c>
       <c r="E26" t="n">
@@ -5134,74 +4988,76 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224313948831</t>
+          <t>https://blog.naver.com/dreamclock33/224325739238</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>창심관 동탄</t>
+          <t>우시이토 문래점</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>동탄맛집</t>
+          <t>문래동 맛집</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>2026. 6. 13.</t>
+          <t>2026. 6. 24.</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224325739238</t>
+          <t>https://blog.naver.com/dreamclock33/224323268859</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>우시이토 문래점</t>
+          <t>낙지마실</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>문래동 맛집</t>
+          <t>보문단지 맛집</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>2026. 6. 24.</t>
+          <t>2026. 6. 22.</t>
         </is>
       </c>
       <c r="E28" t="n">
         <v>1</v>
       </c>
-      <c r="F28" t="inlineStr"/>
+      <c r="F28" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224323268859</t>
+          <t>https://blog.naver.com/dreamclock33/224320953435</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>낙지마실</t>
+          <t>남영동양문 천안점</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>보문단지 맛집</t>
+          <t>불당동 맛집</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>2026. 6. 22.</t>
+          <t>2026. 6. 21.</t>
         </is>
       </c>
       <c r="E29" t="n">
@@ -5212,33 +5068,33 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224320953435</t>
+          <t>https://blog.naver.com/dreamclock33/224313963720</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>남영동양문 천안점</t>
+          <t>워낭 사당본점</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>불당동 맛집</t>
+          <t>사당맛집</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>2026. 6. 21.</t>
+          <t>2026. 6. 14.</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224313963720</t>
+          <t>https://blog.naver.com/dreamclock33/224302834594</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -5253,7 +5109,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>2026. 6. 14.</t>
+          <t>2026. 6. 1.</t>
         </is>
       </c>
       <c r="E31" t="n">
@@ -5264,22 +5120,22 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224302834594</t>
+          <t>https://blog.naver.com/dreamclock33/224324568786</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>워낭 사당본점</t>
+          <t>사당 광안리 사당본점</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>사당맛집</t>
+          <t>사당역 맛집</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>2026. 6. 1.</t>
+          <t>2026. 6. 23.</t>
         </is>
       </c>
       <c r="E32" t="n">
@@ -5290,7 +5146,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224324568786</t>
+          <t>https://blog.naver.com/dreamclock33/224318735799</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -5305,7 +5161,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>2026. 6. 23.</t>
+          <t>2026. 6. 17.</t>
         </is>
       </c>
       <c r="E33" t="n">
@@ -5316,59 +5172,59 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224318735799</t>
+          <t>https://blog.naver.com/dreamclock33/224316861956</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>사당 광안리 사당본점</t>
+          <t>광명대창집 산본점</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>사당역 맛집</t>
+          <t>산본 맛집</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>2026. 6. 17.</t>
+          <t>2026. 6. 15.</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224316861956</t>
+          <t>https://blog.naver.com/dreamclock33/224326686342</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>광명대창집 산본점</t>
+          <t>우와해 선릉본점</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>산본 맛집</t>
+          <t>선릉역 맛집</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>2026. 6. 15.</t>
+          <t>2026. 6. 25.</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224326686342</t>
+          <t>https://blog.naver.com/dreamclock33/224318939548</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -5383,7 +5239,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>2026. 6. 25.</t>
+          <t>2026. 6. 18.</t>
         </is>
       </c>
       <c r="E36" t="n">
@@ -5394,7 +5250,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224318939548</t>
+          <t>https://blog.naver.com/dreamclock33/224310612148</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -5409,7 +5265,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>2026. 6. 18.</t>
+          <t>2026. 6. 10.</t>
         </is>
       </c>
       <c r="E37" t="n">
@@ -5420,7 +5276,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224310612148</t>
+          <t>https://blog.naver.com/dreamclock33/224309471502</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -5435,7 +5291,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>2026. 6. 10.</t>
+          <t>2026. 6. 9.</t>
         </is>
       </c>
       <c r="E38" t="n">
@@ -5446,33 +5302,33 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224309471502</t>
+          <t>https://blog.naver.com/dreamclock33/224316862136</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>우와해 선릉본점</t>
+          <t>우동키노야 성수점</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>선릉역 맛집</t>
+          <t>성수 맛집</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>2026. 6. 9.</t>
+          <t>2026. 6. 15.</t>
         </is>
       </c>
       <c r="E39" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224316862136</t>
+          <t>https://blog.naver.com/dreamclock33/224311781496</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -5487,7 +5343,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>2026. 6. 15.</t>
+          <t>2026. 6. 11.</t>
         </is>
       </c>
       <c r="E40" t="n">
@@ -5498,22 +5354,22 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224311781496</t>
+          <t>https://blog.naver.com/dreamclock33/224325747262</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>우동키노야 성수점</t>
+          <t>고담현불고기 해운대센텀시티점</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>성수 맛집</t>
+          <t>센텀맛집</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>2026. 6. 11.</t>
+          <t>2026. 6. 24.</t>
         </is>
       </c>
       <c r="E41" t="n">
@@ -5524,7 +5380,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224325747262</t>
+          <t>https://blog.naver.com/dreamclock33/224316861777</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -5539,7 +5395,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>2026. 6. 24.</t>
+          <t>2026. 6. 15.</t>
         </is>
       </c>
       <c r="E42" t="n">
@@ -5550,33 +5406,33 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224316861777</t>
+          <t>https://blog.naver.com/dreamclock33/224320956914</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>고담현불고기 해운대센텀시티점</t>
+          <t>청초수물회 속초본점</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>센텀맛집</t>
+          <t>속초맛집</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>2026. 6. 15.</t>
+          <t>2026. 6. 21.</t>
         </is>
       </c>
       <c r="E43" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224320956914</t>
+          <t>https://blog.naver.com/dreamclock33/224313959277</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -5586,12 +5442,12 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>속초맛집</t>
+          <t>속초 물회 맛집</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>2026. 6. 21.</t>
+          <t>2026. 6. 14.</t>
         </is>
       </c>
       <c r="E44" t="n">
@@ -5602,7 +5458,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224313959277</t>
+          <t>https://blog.naver.com/dreamclock33/224275635396</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -5612,12 +5468,12 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>속초 물회 맛집</t>
+          <t>속초 점심 맛집</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>2026. 6. 14.</t>
+          <t>2026. 5. 5.</t>
         </is>
       </c>
       <c r="E45" t="n">
@@ -5628,33 +5484,33 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224275635396</t>
+          <t>https://blog.naver.com/dreamclock33/224317882930</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>청초수물회 속초본점</t>
+          <t>럭키족발 송도점</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>속초 점심 맛집</t>
+          <t>송도 맛집</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>2026. 5. 5.</t>
+          <t>2026. 6. 16.</t>
         </is>
       </c>
       <c r="E46" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224317882930</t>
+          <t>https://blog.naver.com/dreamclock33/224309463239</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -5669,7 +5525,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>2026. 6. 16.</t>
+          <t>2026. 6. 8.</t>
         </is>
       </c>
       <c r="E47" t="n">
@@ -5680,48 +5536,48 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224309463239</t>
+          <t>https://blog.naver.com/dreamclock33/224305766521</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>럭키족발 송도점</t>
+          <t>우동키노야 송도점</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>송도 맛집</t>
+          <t>송도 점심 맛집</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>2026. 6. 8.</t>
+          <t>2026. 6. 4.</t>
         </is>
       </c>
       <c r="E48" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224305766521</t>
+          <t>https://blog.naver.com/dreamclock33/224327987204</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>우동키노야 송도점</t>
+          <t>샤브밀</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>송도 점심 맛집</t>
+          <t>수원맛집</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>2026. 6. 4.</t>
+          <t>2026. 6. 28.</t>
         </is>
       </c>
       <c r="E49" t="n">
@@ -5732,26 +5588,26 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224327987204</t>
+          <t>https://blog.naver.com/dreamclock33/224323273337</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>샤브밀</t>
+          <t>육풍 수원역점</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>수원맛집</t>
+          <t>수원역맛집</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>2026. 6. 28.</t>
+          <t>2026. 6. 22.</t>
         </is>
       </c>
       <c r="E50" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F50" t="inlineStr"/>
     </row>
@@ -5777,7 +5633,7 @@
         </is>
       </c>
       <c r="E51" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F51" t="inlineStr"/>
     </row>
@@ -5831,7 +5687,9 @@
       <c r="E53" t="n">
         <v>1</v>
       </c>
-      <c r="F53" t="inlineStr"/>
+      <c r="F53" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -5867,7 +5725,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>안산 맛</t>
+          <t>부드럽소 안산고잔본점</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -5893,7 +5751,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>라성돌판오리구이</t>
+          <t>라성돌판요리</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -6252,22 +6110,22 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224323273337</t>
+          <t>https://blog.naver.com/dreamclock33/224327991170</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>육풍 수원역</t>
+          <t>창심관 율량점</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>육회 칼비빔면</t>
+          <t>율량동 맛집</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>2026. 6. 22.</t>
+          <t>2026. 6. 28.</t>
         </is>
       </c>
       <c r="E70" t="n">
@@ -6278,33 +6136,33 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224327991170</t>
+          <t>https://blog.naver.com/dreamclock33/224327810468</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>창심관 율량점</t>
+          <t>카츠디나인</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>율량동 맛집</t>
+          <t>이수맛집 추천</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>2026. 6. 28.</t>
+          <t>2026. 6. 27.</t>
         </is>
       </c>
       <c r="E71" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224327810468</t>
+          <t>https://blog.naver.com/dreamclock33/224313034584</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -6319,7 +6177,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>2026. 6. 27.</t>
+          <t>2026. 6. 12.</t>
         </is>
       </c>
       <c r="E72" t="n">
@@ -6330,64 +6188,64 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224313034584</t>
+          <t>https://blog.naver.com/dreamclock33/224327108309</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>카츠디나인</t>
+          <t>샤브가든 종로 타워점</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>이수맛집 추천</t>
+          <t>종로 맛집</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>2026. 6. 12.</t>
+          <t>2026. 6. 26.</t>
         </is>
       </c>
       <c r="E73" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224327108309</t>
+          <t>https://blog.naver.com/dreamclock33/224327995283</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>샤브가든 종로 타워점</t>
+          <t>창심관 율량점</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>종로 맛집</t>
+          <t>청주맛집</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>2026. 6. 26.</t>
+          <t>2026. 6. 28.</t>
         </is>
       </c>
       <c r="E74" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224327995283</t>
+          <t>https://blog.naver.com/dreamclock33/224311773245</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>창심관 율량점</t>
+          <t>아키아키</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -6397,7 +6255,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>2026. 6. 28.</t>
+          <t>2026. 6. 11.</t>
         </is>
       </c>
       <c r="E75" t="n">
@@ -6408,59 +6266,59 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224311773245</t>
+          <t>https://blog.naver.com/dreamclock33/224302825832</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>아키아키</t>
+          <t>창심관</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>청주맛집</t>
+          <t>청주 지웰시티 맛집</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>2026. 6. 11.</t>
+          <t>2026. 6. 1.</t>
         </is>
       </c>
       <c r="E76" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224302825832</t>
+          <t>https://blog.naver.com/dreamclock33/224324620213</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>육질 최상 고기 창심관</t>
+          <t>황토골 충무로역 본점</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>청주 지웰시티 맛집</t>
+          <t>충무로맛집</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>2026. 6. 1.</t>
+          <t>2026. 6. 23.</t>
         </is>
       </c>
       <c r="E77" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224324620213</t>
+          <t>https://blog.naver.com/dreamclock33/224318749373</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -6475,59 +6333,61 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>2026. 6. 23.</t>
+          <t>2026. 6. 17.</t>
         </is>
       </c>
       <c r="E78" t="n">
         <v>2</v>
       </c>
-      <c r="F78" t="inlineStr"/>
+      <c r="F78" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224318749373</t>
+          <t>https://blog.naver.com/dreamclock33/224318944286</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>황토골 충무로역 본점</t>
+          <t>곱마담 아산탕정본점</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>충무로맛집</t>
+          <t>탕정맛집</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>2026. 6. 17.</t>
+          <t>2026. 6. 18.</t>
         </is>
       </c>
       <c r="E79" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224318944286</t>
+          <t>https://blog.naver.com/dreamclock33/224320012596</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>곱마담 아산탕정본점</t>
+          <t>사위식당 판교점</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>탕정맛집</t>
+          <t>판교맛집</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>2026. 6. 18.</t>
+          <t>2026. 6. 19.</t>
         </is>
       </c>
       <c r="E80" t="n">
@@ -6538,33 +6398,33 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224320012596</t>
+          <t>https://blog.naver.com/dreamclock33/224318958749</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>사위식당 판교점</t>
+          <t>대동면옥 올림픽공원직영점</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>판교맛집</t>
+          <t>하남 맛집</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>2026. 6. 19.</t>
+          <t>2026. 6. 18.</t>
         </is>
       </c>
       <c r="E81" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224318958749</t>
+          <t>https://blog.naver.com/dreamclock33/224306893524</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -6579,7 +6439,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>2026. 6. 18.</t>
+          <t>2026. 6. 6.</t>
         </is>
       </c>
       <c r="E82" t="n">
@@ -6590,59 +6450,59 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224306893524</t>
+          <t>https://blog.naver.com/dreamclock33/224320944183</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>대동면옥 올림픽공원직영점</t>
+          <t>신사꽃게당 해운대점</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>하남 맛집</t>
+          <t>해운대 맛집</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>2026. 6. 6.</t>
+          <t>2026. 6. 20.</t>
         </is>
       </c>
       <c r="E83" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224320944183</t>
+          <t>https://blog.naver.com/dreamclock33/224313029267</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>신사꽃게당 해운대점</t>
+          <t>신사 꽃게당</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>해운대 맛집</t>
+          <t>해운대 맛집 추천</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>2026. 6. 20.</t>
+          <t>2026. 6. 12.</t>
         </is>
       </c>
       <c r="E84" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224313029267</t>
+          <t>https://blog.naver.com/dreamclock33/224309460525</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -6657,7 +6517,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>2026. 6. 12.</t>
+          <t>2026. 6. 8.</t>
         </is>
       </c>
       <c r="E85" t="n">
@@ -6668,57 +6528,31 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>https://blog.naver.com/dreamclock33/224309460525</t>
+          <t>https://blog.naver.com/dreamclock33/224305778577</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>신사 꽃게당</t>
+          <t>쟁반집 8292 홍대점</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>해운대 맛집 추천</t>
+          <t>홍대 맛집</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>2026. 6. 8.</t>
+          <t>2026. 6. 5.</t>
         </is>
       </c>
       <c r="E86" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F86" t="inlineStr"/>
     </row>
-    <row r="87">
-      <c r="A87" t="inlineStr">
-        <is>
-          <t>https://blog.naver.com/dreamclock33/224305778577</t>
-        </is>
-      </c>
-      <c r="B87" t="inlineStr">
-        <is>
-          <t>쟁반집 8292 홍대점</t>
-        </is>
-      </c>
-      <c r="C87" t="inlineStr">
-        <is>
-          <t>홍대 맛집</t>
-        </is>
-      </c>
-      <c r="D87" t="inlineStr">
-        <is>
-          <t>2026. 6. 5.</t>
-        </is>
-      </c>
-      <c r="E87" t="n">
-        <v>1</v>
-      </c>
-      <c r="F87" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:E87"/>
+  <autoFilter ref="A1:E86"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6822,7 +6656,9 @@
       <c r="E3" t="n">
         <v>1</v>
       </c>
-      <c r="F3" t="inlineStr"/>
+      <c r="F3" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -8028,7 +7864,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>영등포 맛</t>
+          <t>호우양꼬치</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -9711,7 +9547,9 @@
       <c r="E41" t="n">
         <v>1</v>
       </c>
-      <c r="F41" t="inlineStr"/>
+      <c r="F41" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">

</xml_diff>